<commit_message>
Updated Coal Capacitu factor for preexixting power plant
</commit_message>
<xml_diff>
--- a/InputData/elec/BECF/BAU Expected Capacity Factors.xlsx
+++ b/InputData/elec/BECF/BAU Expected Capacity Factors.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Postdoc Projects/eps-indonesia-cpl/InputData/elec/BECF/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85CFDB6A-613F-F74A-AF36-251C24C31E36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8940C2D2-088D-7842-BAAF-765B015382C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21360" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21360" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="177">
   <si>
     <t>BAU Expected Capacity Factors</t>
   </si>
@@ -622,6 +622,9 @@
   </si>
   <si>
     <t> In 2021, the global median capacity factor was 85.6%, in line with recent years. Pressurized water reactors (PWR) and pressurized heavy water moderated, and cooled reactors (PHWR) have been the best performing reactors since 2011, with median capacity factors of 82% and 81%, respectively.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preexisting coal power </t>
   </si>
 </sst>
 </file>
@@ -1220,6 +1223,15 @@
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1230,23 +1242,29 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1263,30 +1281,15 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1622,16 +1625,16 @@
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="84" t="s">
+      <c r="B3" s="87" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="85"/>
-      <c r="D3" s="85"/>
-      <c r="E3" s="85"/>
-      <c r="F3" s="85"/>
-      <c r="G3" s="85"/>
-      <c r="H3" s="85"/>
-      <c r="I3" s="86"/>
+      <c r="C3" s="88"/>
+      <c r="D3" s="88"/>
+      <c r="E3" s="88"/>
+      <c r="F3" s="88"/>
+      <c r="G3" s="88"/>
+      <c r="H3" s="88"/>
+      <c r="I3" s="89"/>
     </row>
     <row r="4" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
@@ -1871,7 +1874,7 @@
     </row>
     <row r="46" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2"/>
-      <c r="B46" s="110">
+      <c r="B46" s="84">
         <v>2021</v>
       </c>
     </row>
@@ -1906,141 +1909,141 @@
       <c r="B52" s="2"/>
     </row>
     <row r="53" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B53" s="87" t="s">
+      <c r="B53" s="90" t="s">
         <v>8</v>
       </c>
-      <c r="C53" s="88"/>
-      <c r="D53" s="88"/>
-      <c r="E53" s="88"/>
-      <c r="F53" s="88"/>
-      <c r="G53" s="88"/>
-      <c r="H53" s="88"/>
-      <c r="I53" s="88"/>
+      <c r="C53" s="91"/>
+      <c r="D53" s="91"/>
+      <c r="E53" s="91"/>
+      <c r="F53" s="91"/>
+      <c r="G53" s="91"/>
+      <c r="H53" s="91"/>
+      <c r="I53" s="91"/>
     </row>
     <row r="54" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B54" s="88"/>
-      <c r="C54" s="88"/>
-      <c r="D54" s="88"/>
-      <c r="E54" s="88"/>
-      <c r="F54" s="88"/>
-      <c r="G54" s="88"/>
-      <c r="H54" s="88"/>
-      <c r="I54" s="88"/>
+      <c r="B54" s="91"/>
+      <c r="C54" s="91"/>
+      <c r="D54" s="91"/>
+      <c r="E54" s="91"/>
+      <c r="F54" s="91"/>
+      <c r="G54" s="91"/>
+      <c r="H54" s="91"/>
+      <c r="I54" s="91"/>
     </row>
     <row r="55" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B55" s="88"/>
-      <c r="C55" s="88"/>
-      <c r="D55" s="88"/>
-      <c r="E55" s="88"/>
-      <c r="F55" s="88"/>
-      <c r="G55" s="88"/>
-      <c r="H55" s="88"/>
-      <c r="I55" s="88"/>
+      <c r="B55" s="91"/>
+      <c r="C55" s="91"/>
+      <c r="D55" s="91"/>
+      <c r="E55" s="91"/>
+      <c r="F55" s="91"/>
+      <c r="G55" s="91"/>
+      <c r="H55" s="91"/>
+      <c r="I55" s="91"/>
     </row>
     <row r="56" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B56" s="88"/>
-      <c r="C56" s="88"/>
-      <c r="D56" s="88"/>
-      <c r="E56" s="88"/>
-      <c r="F56" s="88"/>
-      <c r="G56" s="88"/>
-      <c r="H56" s="88"/>
-      <c r="I56" s="88"/>
+      <c r="B56" s="91"/>
+      <c r="C56" s="91"/>
+      <c r="D56" s="91"/>
+      <c r="E56" s="91"/>
+      <c r="F56" s="91"/>
+      <c r="G56" s="91"/>
+      <c r="H56" s="91"/>
+      <c r="I56" s="91"/>
     </row>
     <row r="57" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B57" s="88"/>
-      <c r="C57" s="88"/>
-      <c r="D57" s="88"/>
-      <c r="E57" s="88"/>
-      <c r="F57" s="88"/>
-      <c r="G57" s="88"/>
-      <c r="H57" s="88"/>
-      <c r="I57" s="88"/>
+      <c r="B57" s="91"/>
+      <c r="C57" s="91"/>
+      <c r="D57" s="91"/>
+      <c r="E57" s="91"/>
+      <c r="F57" s="91"/>
+      <c r="G57" s="91"/>
+      <c r="H57" s="91"/>
+      <c r="I57" s="91"/>
     </row>
     <row r="58" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B58" s="88"/>
-      <c r="C58" s="88"/>
-      <c r="D58" s="88"/>
-      <c r="E58" s="88"/>
-      <c r="F58" s="88"/>
-      <c r="G58" s="88"/>
-      <c r="H58" s="88"/>
-      <c r="I58" s="88"/>
+      <c r="B58" s="91"/>
+      <c r="C58" s="91"/>
+      <c r="D58" s="91"/>
+      <c r="E58" s="91"/>
+      <c r="F58" s="91"/>
+      <c r="G58" s="91"/>
+      <c r="H58" s="91"/>
+      <c r="I58" s="91"/>
     </row>
     <row r="59" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B59" s="88"/>
-      <c r="C59" s="88"/>
-      <c r="D59" s="88"/>
-      <c r="E59" s="88"/>
-      <c r="F59" s="88"/>
-      <c r="G59" s="88"/>
-      <c r="H59" s="88"/>
-      <c r="I59" s="88"/>
+      <c r="B59" s="91"/>
+      <c r="C59" s="91"/>
+      <c r="D59" s="91"/>
+      <c r="E59" s="91"/>
+      <c r="F59" s="91"/>
+      <c r="G59" s="91"/>
+      <c r="H59" s="91"/>
+      <c r="I59" s="91"/>
     </row>
     <row r="60" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B60" s="88"/>
-      <c r="C60" s="88"/>
-      <c r="D60" s="88"/>
-      <c r="E60" s="88"/>
-      <c r="F60" s="88"/>
-      <c r="G60" s="88"/>
-      <c r="H60" s="88"/>
-      <c r="I60" s="88"/>
+      <c r="B60" s="91"/>
+      <c r="C60" s="91"/>
+      <c r="D60" s="91"/>
+      <c r="E60" s="91"/>
+      <c r="F60" s="91"/>
+      <c r="G60" s="91"/>
+      <c r="H60" s="91"/>
+      <c r="I60" s="91"/>
     </row>
     <row r="61" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B61" s="88"/>
-      <c r="C61" s="88"/>
-      <c r="D61" s="88"/>
-      <c r="E61" s="88"/>
-      <c r="F61" s="88"/>
-      <c r="G61" s="88"/>
-      <c r="H61" s="88"/>
-      <c r="I61" s="88"/>
+      <c r="B61" s="91"/>
+      <c r="C61" s="91"/>
+      <c r="D61" s="91"/>
+      <c r="E61" s="91"/>
+      <c r="F61" s="91"/>
+      <c r="G61" s="91"/>
+      <c r="H61" s="91"/>
+      <c r="I61" s="91"/>
     </row>
     <row r="62" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B62" s="88"/>
-      <c r="C62" s="88"/>
-      <c r="D62" s="88"/>
-      <c r="E62" s="88"/>
-      <c r="F62" s="88"/>
-      <c r="G62" s="88"/>
-      <c r="H62" s="88"/>
-      <c r="I62" s="88"/>
+      <c r="B62" s="91"/>
+      <c r="C62" s="91"/>
+      <c r="D62" s="91"/>
+      <c r="E62" s="91"/>
+      <c r="F62" s="91"/>
+      <c r="G62" s="91"/>
+      <c r="H62" s="91"/>
+      <c r="I62" s="91"/>
     </row>
     <row r="63" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B63" s="88"/>
-      <c r="C63" s="88"/>
-      <c r="D63" s="88"/>
-      <c r="E63" s="88"/>
-      <c r="F63" s="88"/>
-      <c r="G63" s="88"/>
-      <c r="H63" s="88"/>
-      <c r="I63" s="88"/>
+      <c r="B63" s="91"/>
+      <c r="C63" s="91"/>
+      <c r="D63" s="91"/>
+      <c r="E63" s="91"/>
+      <c r="F63" s="91"/>
+      <c r="G63" s="91"/>
+      <c r="H63" s="91"/>
+      <c r="I63" s="91"/>
     </row>
     <row r="64" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B64" s="88"/>
-      <c r="C64" s="88"/>
-      <c r="D64" s="88"/>
-      <c r="E64" s="88"/>
-      <c r="F64" s="88"/>
-      <c r="G64" s="88"/>
-      <c r="H64" s="88"/>
-      <c r="I64" s="88"/>
+      <c r="B64" s="91"/>
+      <c r="C64" s="91"/>
+      <c r="D64" s="91"/>
+      <c r="E64" s="91"/>
+      <c r="F64" s="91"/>
+      <c r="G64" s="91"/>
+      <c r="H64" s="91"/>
+      <c r="I64" s="91"/>
     </row>
     <row r="65" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B65" s="88"/>
-      <c r="C65" s="88"/>
-      <c r="D65" s="88"/>
-      <c r="E65" s="88"/>
-      <c r="F65" s="88"/>
-      <c r="G65" s="88"/>
-      <c r="H65" s="88"/>
-      <c r="I65" s="88"/>
+      <c r="B65" s="91"/>
+      <c r="C65" s="91"/>
+      <c r="D65" s="91"/>
+      <c r="E65" s="91"/>
+      <c r="F65" s="91"/>
+      <c r="G65" s="91"/>
+      <c r="H65" s="91"/>
+      <c r="I65" s="91"/>
     </row>
     <row r="66" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="67" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="68" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B68" s="111" t="s">
+      <c r="B68" s="85" t="s">
         <v>175</v>
       </c>
     </row>
@@ -3051,11 +3054,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="100" t="s">
+      <c r="A1" s="105" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="85"/>
-      <c r="C1" s="86"/>
+      <c r="B1" s="88"/>
+      <c r="C1" s="89"/>
       <c r="D1" s="1" t="s">
         <v>10</v>
       </c>
@@ -3066,14 +3069,14 @@
       <c r="C2" s="5"/>
     </row>
     <row r="3" spans="1:30" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="101" t="s">
+      <c r="A3" s="106" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="90"/>
-      <c r="C3" s="102" t="s">
+      <c r="B3" s="93"/>
+      <c r="C3" s="107" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="90"/>
+      <c r="D3" s="93"/>
       <c r="E3" s="6" t="s">
         <v>13</v>
       </c>
@@ -3144,14 +3147,14 @@
       </c>
     </row>
     <row r="4" spans="1:30" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="103" t="s">
+      <c r="A4" s="108" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="92"/>
-      <c r="C4" s="104" t="s">
+      <c r="B4" s="99"/>
+      <c r="C4" s="92" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="90"/>
+      <c r="D4" s="93"/>
       <c r="E4" s="12" t="s">
         <v>25</v>
       </c>
@@ -3233,12 +3236,12 @@
       </c>
     </row>
     <row r="5" spans="1:30" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="93"/>
-      <c r="B5" s="94"/>
-      <c r="C5" s="104" t="s">
+      <c r="A5" s="102"/>
+      <c r="B5" s="103"/>
+      <c r="C5" s="92" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="90"/>
+      <c r="D5" s="93"/>
       <c r="E5" s="12">
         <v>3</v>
       </c>
@@ -3317,14 +3320,14 @@
       </c>
     </row>
     <row r="6" spans="1:30" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="89" t="s">
+      <c r="A6" s="109" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="90"/>
-      <c r="C6" s="104" t="s">
+      <c r="B6" s="93"/>
+      <c r="C6" s="92" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="90"/>
+      <c r="D6" s="93"/>
       <c r="E6" s="12" t="s">
         <v>28</v>
       </c>
@@ -3403,14 +3406,14 @@
       </c>
     </row>
     <row r="7" spans="1:30" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="91" t="s">
+      <c r="A7" s="110" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="92"/>
-      <c r="C7" s="104" t="s">
+      <c r="B7" s="99"/>
+      <c r="C7" s="92" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="90"/>
+      <c r="D7" s="93"/>
       <c r="E7" s="12" t="s">
         <v>28</v>
       </c>
@@ -3489,12 +3492,12 @@
       </c>
     </row>
     <row r="8" spans="1:30" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="93"/>
-      <c r="B8" s="94"/>
-      <c r="C8" s="104" t="s">
+      <c r="A8" s="102"/>
+      <c r="B8" s="103"/>
+      <c r="C8" s="92" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="90"/>
+      <c r="D8" s="93"/>
       <c r="E8" s="12">
         <v>1</v>
       </c>
@@ -3573,14 +3576,14 @@
       </c>
     </row>
     <row r="9" spans="1:30" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="95" t="s">
+      <c r="A9" s="111" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="92"/>
-      <c r="C9" s="104" t="s">
+      <c r="B9" s="99"/>
+      <c r="C9" s="92" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="90"/>
+      <c r="D9" s="93"/>
       <c r="E9" s="12" t="s">
         <v>32</v>
       </c>
@@ -3659,12 +3662,12 @@
       </c>
     </row>
     <row r="10" spans="1:30" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="96"/>
-      <c r="B10" s="97"/>
-      <c r="C10" s="104" t="s">
+      <c r="A10" s="100"/>
+      <c r="B10" s="101"/>
+      <c r="C10" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="D10" s="90"/>
+      <c r="D10" s="93"/>
       <c r="E10" s="12" t="s">
         <v>28</v>
       </c>
@@ -3743,12 +3746,12 @@
       </c>
     </row>
     <row r="11" spans="1:30" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="96"/>
-      <c r="B11" s="97"/>
-      <c r="C11" s="104" t="s">
+      <c r="A11" s="100"/>
+      <c r="B11" s="101"/>
+      <c r="C11" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="90"/>
+      <c r="D11" s="93"/>
       <c r="E11" s="12" t="s">
         <v>28</v>
       </c>
@@ -3827,12 +3830,12 @@
       </c>
     </row>
     <row r="12" spans="1:30" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="93"/>
-      <c r="B12" s="94"/>
-      <c r="C12" s="104" t="s">
+      <c r="A12" s="102"/>
+      <c r="B12" s="103"/>
+      <c r="C12" s="92" t="s">
         <v>35</v>
       </c>
-      <c r="D12" s="90"/>
+      <c r="D12" s="93"/>
       <c r="E12" s="12" t="s">
         <v>28</v>
       </c>
@@ -3877,14 +3880,14 @@
       </c>
     </row>
     <row r="13" spans="1:30" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="95" t="s">
+      <c r="A13" s="111" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="92"/>
-      <c r="C13" s="104" t="s">
+      <c r="B13" s="99"/>
+      <c r="C13" s="92" t="s">
         <v>36</v>
       </c>
-      <c r="D13" s="90"/>
+      <c r="D13" s="93"/>
       <c r="E13" s="12" t="s">
         <v>37</v>
       </c>
@@ -3962,12 +3965,12 @@
       </c>
     </row>
     <row r="14" spans="1:30" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="93"/>
-      <c r="B14" s="94"/>
-      <c r="C14" s="104" t="s">
+      <c r="A14" s="102"/>
+      <c r="B14" s="103"/>
+      <c r="C14" s="92" t="s">
         <v>38</v>
       </c>
-      <c r="D14" s="90"/>
+      <c r="D14" s="93"/>
       <c r="E14" s="12">
         <v>3</v>
       </c>
@@ -4206,14 +4209,14 @@
       </c>
     </row>
     <row r="17" spans="1:30" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="95" t="s">
+      <c r="A17" s="111" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="92"/>
-      <c r="C17" s="104" t="s">
+      <c r="B17" s="99"/>
+      <c r="C17" s="92" t="s">
         <v>39</v>
       </c>
-      <c r="D17" s="90"/>
+      <c r="D17" s="93"/>
       <c r="E17" s="12" t="s">
         <v>28</v>
       </c>
@@ -4253,12 +4256,12 @@
       </c>
     </row>
     <row r="18" spans="1:30" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="93"/>
-      <c r="B18" s="94"/>
-      <c r="C18" s="104" t="s">
+      <c r="A18" s="102"/>
+      <c r="B18" s="103"/>
+      <c r="C18" s="92" t="s">
         <v>40</v>
       </c>
-      <c r="D18" s="90"/>
+      <c r="D18" s="93"/>
       <c r="E18" s="12">
         <v>1</v>
       </c>
@@ -4304,11 +4307,11 @@
       <c r="A19" s="98" t="s">
         <v>21</v>
       </c>
-      <c r="B19" s="92"/>
-      <c r="C19" s="104" t="s">
+      <c r="B19" s="99"/>
+      <c r="C19" s="92" t="s">
         <v>42</v>
       </c>
-      <c r="D19" s="90"/>
+      <c r="D19" s="93"/>
       <c r="E19" s="12" t="s">
         <v>37</v>
       </c>
@@ -4361,12 +4364,12 @@
       </c>
     </row>
     <row r="20" spans="1:30" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="96"/>
-      <c r="B20" s="97"/>
-      <c r="C20" s="104" t="s">
+      <c r="A20" s="100"/>
+      <c r="B20" s="101"/>
+      <c r="C20" s="92" t="s">
         <v>47</v>
       </c>
-      <c r="D20" s="90"/>
+      <c r="D20" s="93"/>
       <c r="E20" s="12" t="s">
         <v>37</v>
       </c>
@@ -4425,12 +4428,12 @@
       </c>
     </row>
     <row r="21" spans="1:30" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="93"/>
-      <c r="B21" s="94"/>
-      <c r="C21" s="104" t="s">
+      <c r="A21" s="102"/>
+      <c r="B21" s="103"/>
+      <c r="C21" s="92" t="s">
         <v>48</v>
       </c>
-      <c r="D21" s="90"/>
+      <c r="D21" s="93"/>
       <c r="E21" s="12">
         <v>2</v>
       </c>
@@ -4489,14 +4492,14 @@
       </c>
     </row>
     <row r="22" spans="1:30" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="99" t="s">
+      <c r="A22" s="104" t="s">
         <v>22</v>
       </c>
-      <c r="B22" s="90"/>
-      <c r="C22" s="104" t="s">
+      <c r="B22" s="93"/>
+      <c r="C22" s="92" t="s">
         <v>49</v>
       </c>
-      <c r="D22" s="90"/>
+      <c r="D22" s="93"/>
       <c r="E22" s="12">
         <v>2</v>
       </c>
@@ -4524,11 +4527,11 @@
       <c r="A23" s="98" t="s">
         <v>23</v>
       </c>
-      <c r="B23" s="92"/>
-      <c r="C23" s="104" t="s">
+      <c r="B23" s="99"/>
+      <c r="C23" s="92" t="s">
         <v>50</v>
       </c>
-      <c r="D23" s="90"/>
+      <c r="D23" s="93"/>
       <c r="E23" s="12" t="s">
         <v>28</v>
       </c>
@@ -4553,12 +4556,12 @@
       </c>
     </row>
     <row r="24" spans="1:30" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="96"/>
-      <c r="B24" s="97"/>
-      <c r="C24" s="105" t="s">
+      <c r="A24" s="100"/>
+      <c r="B24" s="101"/>
+      <c r="C24" s="97" t="s">
         <v>51</v>
       </c>
-      <c r="D24" s="90"/>
+      <c r="D24" s="93"/>
       <c r="E24" s="12">
         <v>3</v>
       </c>
@@ -4616,12 +4619,12 @@
       </c>
     </row>
     <row r="25" spans="1:30" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="96"/>
-      <c r="B25" s="97"/>
-      <c r="C25" s="105" t="s">
+      <c r="A25" s="100"/>
+      <c r="B25" s="101"/>
+      <c r="C25" s="97" t="s">
         <v>52</v>
       </c>
-      <c r="D25" s="90"/>
+      <c r="D25" s="93"/>
       <c r="E25" s="12">
         <v>3</v>
       </c>
@@ -4649,12 +4652,12 @@
       </c>
     </row>
     <row r="26" spans="1:30" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="96"/>
-      <c r="B26" s="97"/>
-      <c r="C26" s="105" t="s">
+      <c r="A26" s="100"/>
+      <c r="B26" s="101"/>
+      <c r="C26" s="97" t="s">
         <v>53</v>
       </c>
-      <c r="D26" s="90"/>
+      <c r="D26" s="93"/>
       <c r="E26" s="12">
         <v>3</v>
       </c>
@@ -4682,12 +4685,12 @@
       </c>
     </row>
     <row r="27" spans="1:30" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="93"/>
-      <c r="B27" s="94"/>
-      <c r="C27" s="104" t="s">
+      <c r="A27" s="102"/>
+      <c r="B27" s="103"/>
+      <c r="C27" s="92" t="s">
         <v>38</v>
       </c>
-      <c r="D27" s="90"/>
+      <c r="D27" s="93"/>
       <c r="E27" s="12">
         <v>3</v>
       </c>
@@ -4858,12 +4861,12 @@
       </c>
     </row>
     <row r="35" spans="1:30" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F35" s="106" t="s">
+      <c r="F35" s="94" t="s">
         <v>55</v>
       </c>
-      <c r="G35" s="88"/>
-      <c r="H35" s="88"/>
-      <c r="I35" s="88"/>
+      <c r="G35" s="91"/>
+      <c r="H35" s="91"/>
+      <c r="I35" s="91"/>
     </row>
     <row r="36" spans="1:30" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="27" t="s">
@@ -5563,12 +5566,12 @@
       <c r="D52" s="32"/>
     </row>
     <row r="53" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="107" t="s">
+      <c r="A53" s="95" t="s">
         <v>67</v>
       </c>
-      <c r="B53" s="85"/>
-      <c r="C53" s="85"/>
-      <c r="D53" s="86"/>
+      <c r="B53" s="88"/>
+      <c r="C53" s="88"/>
+      <c r="D53" s="89"/>
       <c r="E53" s="26" t="s">
         <v>10</v>
       </c>
@@ -5578,11 +5581,11 @@
       <c r="B54" s="37"/>
       <c r="C54" s="37"/>
       <c r="D54" s="37"/>
-      <c r="F54" s="106" t="s">
+      <c r="F54" s="94" t="s">
         <v>55</v>
       </c>
-      <c r="G54" s="88"/>
-      <c r="H54" s="88"/>
+      <c r="G54" s="91"/>
+      <c r="H54" s="91"/>
     </row>
     <row r="55" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="27" t="s">
@@ -6370,12 +6373,12 @@
     </row>
     <row r="69" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="70" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="108" t="s">
+      <c r="A70" s="96" t="s">
         <v>71</v>
       </c>
-      <c r="B70" s="85"/>
-      <c r="C70" s="85"/>
-      <c r="D70" s="86"/>
+      <c r="B70" s="88"/>
+      <c r="C70" s="88"/>
+      <c r="D70" s="89"/>
       <c r="E70" s="26" t="s">
         <v>10</v>
       </c>
@@ -7846,23 +7849,11 @@
     <row r="1012" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="F35:I35"/>
-    <mergeCell ref="F54:H54"/>
-    <mergeCell ref="A53:D53"/>
-    <mergeCell ref="A70:D70"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:B8"/>
+    <mergeCell ref="A9:B12"/>
+    <mergeCell ref="A13:B14"/>
+    <mergeCell ref="A17:B18"/>
     <mergeCell ref="A19:B21"/>
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="A23:B27"/>
@@ -7879,11 +7870,23 @@
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="C12:D12"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A7:B8"/>
-    <mergeCell ref="A9:B12"/>
-    <mergeCell ref="A13:B14"/>
-    <mergeCell ref="A17:B18"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="F35:I35"/>
+    <mergeCell ref="F54:H54"/>
+    <mergeCell ref="A53:D53"/>
+    <mergeCell ref="A70:D70"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -7905,11 +7908,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="100" t="s">
+      <c r="A1" s="105" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="85"/>
-      <c r="C1" s="86"/>
+      <c r="B1" s="88"/>
+      <c r="C1" s="89"/>
       <c r="D1" s="1" t="s">
         <v>78</v>
       </c>
@@ -7920,14 +7923,14 @@
       <c r="C2" s="5"/>
     </row>
     <row r="3" spans="1:26" ht="39" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="101" t="s">
+      <c r="A3" s="106" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="90"/>
-      <c r="C3" s="102" t="s">
+      <c r="B3" s="93"/>
+      <c r="C3" s="107" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="90"/>
+      <c r="D3" s="93"/>
       <c r="E3" s="6" t="s">
         <v>13</v>
       </c>
@@ -7963,14 +7966,14 @@
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="103" t="s">
+      <c r="A4" s="108" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="92"/>
-      <c r="C4" s="99" t="s">
+      <c r="B4" s="99"/>
+      <c r="C4" s="104" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="90"/>
+      <c r="D4" s="93"/>
       <c r="E4" s="12" t="s">
         <v>28</v>
       </c>
@@ -8015,12 +8018,12 @@
       </c>
     </row>
     <row r="5" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="96"/>
-      <c r="B5" s="97"/>
-      <c r="C5" s="104" t="s">
+      <c r="A5" s="100"/>
+      <c r="B5" s="101"/>
+      <c r="C5" s="92" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="90"/>
+      <c r="D5" s="93"/>
       <c r="E5" s="12" t="s">
         <v>28</v>
       </c>
@@ -8065,12 +8068,12 @@
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="93"/>
-      <c r="B6" s="94"/>
-      <c r="C6" s="104" t="s">
+      <c r="A6" s="102"/>
+      <c r="B6" s="103"/>
+      <c r="C6" s="92" t="s">
         <v>79</v>
       </c>
-      <c r="D6" s="90"/>
+      <c r="D6" s="93"/>
       <c r="E6" s="12">
         <v>1</v>
       </c>
@@ -8115,14 +8118,14 @@
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="89" t="s">
+      <c r="A7" s="109" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="90"/>
-      <c r="C7" s="109" t="s">
+      <c r="B7" s="93"/>
+      <c r="C7" s="112" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="90"/>
+      <c r="D7" s="93"/>
       <c r="E7" s="12">
         <v>1</v>
       </c>
@@ -8167,14 +8170,14 @@
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="91" t="s">
+      <c r="A8" s="110" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="92"/>
-      <c r="C8" s="109" t="s">
+      <c r="B8" s="99"/>
+      <c r="C8" s="112" t="s">
         <v>80</v>
       </c>
-      <c r="D8" s="90"/>
+      <c r="D8" s="93"/>
       <c r="E8" s="12">
         <v>1</v>
       </c>
@@ -8219,12 +8222,12 @@
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="96"/>
-      <c r="B9" s="97"/>
-      <c r="C9" s="109" t="s">
+      <c r="A9" s="100"/>
+      <c r="B9" s="101"/>
+      <c r="C9" s="112" t="s">
         <v>29</v>
       </c>
-      <c r="D9" s="90"/>
+      <c r="D9" s="93"/>
       <c r="E9" s="12">
         <v>1</v>
       </c>
@@ -8269,12 +8272,12 @@
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="93"/>
-      <c r="B10" s="94"/>
-      <c r="C10" s="104" t="s">
+      <c r="A10" s="102"/>
+      <c r="B10" s="103"/>
+      <c r="C10" s="92" t="s">
         <v>50</v>
       </c>
-      <c r="D10" s="90"/>
+      <c r="D10" s="93"/>
       <c r="E10" s="12">
         <v>1</v>
       </c>
@@ -8330,14 +8333,14 @@
       <c r="Z10" s="2"/>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="95" t="s">
+      <c r="A11" s="111" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="92"/>
-      <c r="C11" s="109" t="s">
+      <c r="B11" s="99"/>
+      <c r="C11" s="112" t="s">
         <v>81</v>
       </c>
-      <c r="D11" s="90"/>
+      <c r="D11" s="93"/>
       <c r="E11" s="12">
         <v>1</v>
       </c>
@@ -8382,12 +8385,12 @@
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="96"/>
-      <c r="B12" s="97"/>
-      <c r="C12" s="109" t="s">
+      <c r="A12" s="100"/>
+      <c r="B12" s="101"/>
+      <c r="C12" s="112" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="90"/>
+      <c r="D12" s="93"/>
       <c r="E12" s="12">
         <v>1</v>
       </c>
@@ -8432,12 +8435,12 @@
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="96"/>
-      <c r="B13" s="97"/>
-      <c r="C13" s="109" t="s">
+      <c r="A13" s="100"/>
+      <c r="B13" s="101"/>
+      <c r="C13" s="112" t="s">
         <v>82</v>
       </c>
-      <c r="D13" s="90"/>
+      <c r="D13" s="93"/>
       <c r="E13" s="12">
         <v>1</v>
       </c>
@@ -8482,12 +8485,12 @@
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="93"/>
-      <c r="B14" s="94"/>
-      <c r="C14" s="109" t="s">
+      <c r="A14" s="102"/>
+      <c r="B14" s="103"/>
+      <c r="C14" s="112" t="s">
         <v>35</v>
       </c>
-      <c r="D14" s="90"/>
+      <c r="D14" s="93"/>
       <c r="E14" s="12">
         <v>1</v>
       </c>
@@ -8624,25 +8627,25 @@
       </c>
     </row>
     <row r="17" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="95" t="s">
+      <c r="A17" s="111" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="92"/>
-      <c r="C17" s="109" t="s">
+      <c r="B17" s="99"/>
+      <c r="C17" s="112" t="s">
         <v>36</v>
       </c>
-      <c r="D17" s="90"/>
+      <c r="D17" s="93"/>
       <c r="E17" s="12" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="93"/>
-      <c r="B18" s="94"/>
-      <c r="C18" s="109" t="s">
+      <c r="A18" s="102"/>
+      <c r="B18" s="103"/>
+      <c r="C18" s="112" t="s">
         <v>38</v>
       </c>
-      <c r="D18" s="90"/>
+      <c r="D18" s="93"/>
       <c r="E18" s="12">
         <v>2</v>
       </c>
@@ -8651,14 +8654,14 @@
       </c>
     </row>
     <row r="19" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="95" t="s">
+      <c r="A19" s="111" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="92"/>
-      <c r="C19" s="109" t="s">
+      <c r="B19" s="99"/>
+      <c r="C19" s="112" t="s">
         <v>84</v>
       </c>
-      <c r="D19" s="90"/>
+      <c r="D19" s="93"/>
       <c r="E19" s="12">
         <v>1</v>
       </c>
@@ -8676,12 +8679,12 @@
       </c>
     </row>
     <row r="20" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="93"/>
-      <c r="B20" s="94"/>
-      <c r="C20" s="104" t="s">
+      <c r="A20" s="102"/>
+      <c r="B20" s="103"/>
+      <c r="C20" s="92" t="s">
         <v>85</v>
       </c>
-      <c r="D20" s="90"/>
+      <c r="D20" s="93"/>
       <c r="E20" s="12">
         <v>1</v>
       </c>
@@ -8705,11 +8708,11 @@
       <c r="A21" s="98" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="92"/>
-      <c r="C21" s="104" t="s">
+      <c r="B21" s="99"/>
+      <c r="C21" s="92" t="s">
         <v>47</v>
       </c>
-      <c r="D21" s="90"/>
+      <c r="D21" s="93"/>
       <c r="E21" s="12" t="s">
         <v>28</v>
       </c>
@@ -8730,8 +8733,8 @@
       </c>
     </row>
     <row r="22" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="93"/>
-      <c r="B22" s="94"/>
+      <c r="A22" s="102"/>
+      <c r="B22" s="103"/>
       <c r="C22" s="21" t="s">
         <v>42</v>
       </c>
@@ -8756,14 +8759,14 @@
       </c>
     </row>
     <row r="23" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="99" t="s">
+      <c r="A23" s="104" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="90"/>
-      <c r="C23" s="104" t="s">
+      <c r="B23" s="93"/>
+      <c r="C23" s="92" t="s">
         <v>49</v>
       </c>
-      <c r="D23" s="90"/>
+      <c r="D23" s="93"/>
       <c r="E23" s="12">
         <v>1</v>
       </c>
@@ -8787,11 +8790,11 @@
       <c r="A24" s="98" t="s">
         <v>23</v>
       </c>
-      <c r="B24" s="92"/>
-      <c r="C24" s="104" t="s">
+      <c r="B24" s="99"/>
+      <c r="C24" s="92" t="s">
         <v>50</v>
       </c>
-      <c r="D24" s="90"/>
+      <c r="D24" s="93"/>
       <c r="E24" s="12">
         <v>1</v>
       </c>
@@ -8812,12 +8815,12 @@
       </c>
     </row>
     <row r="25" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="96"/>
-      <c r="B25" s="97"/>
-      <c r="C25" s="109" t="s">
+      <c r="A25" s="100"/>
+      <c r="B25" s="101"/>
+      <c r="C25" s="112" t="s">
         <v>53</v>
       </c>
-      <c r="D25" s="90"/>
+      <c r="D25" s="93"/>
       <c r="E25" s="12">
         <v>2</v>
       </c>
@@ -8838,12 +8841,12 @@
       </c>
     </row>
     <row r="26" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="96"/>
-      <c r="B26" s="97"/>
-      <c r="C26" s="105" t="s">
+      <c r="A26" s="100"/>
+      <c r="B26" s="101"/>
+      <c r="C26" s="97" t="s">
         <v>51</v>
       </c>
-      <c r="D26" s="90"/>
+      <c r="D26" s="93"/>
       <c r="E26" s="12">
         <v>2</v>
       </c>
@@ -8864,12 +8867,12 @@
       </c>
     </row>
     <row r="27" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="96"/>
-      <c r="B27" s="97"/>
-      <c r="C27" s="105" t="s">
+      <c r="A27" s="100"/>
+      <c r="B27" s="101"/>
+      <c r="C27" s="97" t="s">
         <v>52</v>
       </c>
-      <c r="D27" s="90"/>
+      <c r="D27" s="93"/>
       <c r="E27" s="12">
         <v>2</v>
       </c>
@@ -8890,12 +8893,12 @@
       </c>
     </row>
     <row r="28" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="93"/>
-      <c r="B28" s="94"/>
-      <c r="C28" s="104" t="s">
+      <c r="A28" s="102"/>
+      <c r="B28" s="103"/>
+      <c r="C28" s="92" t="s">
         <v>38</v>
       </c>
-      <c r="D28" s="90"/>
+      <c r="D28" s="93"/>
       <c r="E28" s="12">
         <v>2</v>
       </c>
@@ -10940,22 +10943,13 @@
     <row r="1010" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="A21:B22"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="A24:B28"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="A17:B18"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="A19:B20"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="A4:B6"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C6:D6"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="C12:D12"/>
     <mergeCell ref="C13:D13"/>
@@ -10967,13 +10961,22 @@
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="A11:B14"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="A4:B6"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="A17:B18"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="A19:B20"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="A21:B22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="A24:B28"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C26:D26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -18929,23 +18932,29 @@
     <col min="14" max="14" width="134.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="65" t="s">
         <v>150</v>
       </c>
       <c r="B1" s="65" t="s">
         <v>151</v>
       </c>
+      <c r="C1" s="65" t="s">
+        <v>176</v>
+      </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="55" t="s">
         <v>126</v>
       </c>
       <c r="B2">
         <v>0.65</v>
       </c>
+      <c r="C2">
+        <v>0.49</v>
+      </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="54" t="s">
         <v>127</v>
       </c>
@@ -18953,7 +18962,7 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="54" t="s">
         <v>128</v>
       </c>
@@ -18962,7 +18971,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="54" t="s">
         <v>15</v>
       </c>
@@ -18970,7 +18979,7 @@
         <v>0.37</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="54" t="s">
         <v>129</v>
       </c>
@@ -18978,7 +18987,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="54" t="s">
         <v>23</v>
       </c>
@@ -18986,7 +18995,7 @@
         <v>0.18</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="54" t="s">
         <v>130</v>
       </c>
@@ -18995,7 +19004,7 @@
         <v>0.18</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="54" t="s">
         <v>21</v>
       </c>
@@ -19003,7 +19012,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="54" t="s">
         <v>16</v>
       </c>
@@ -19011,7 +19020,7 @@
         <v>0.82</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="54" t="s">
         <v>131</v>
       </c>
@@ -19019,7 +19028,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="54" t="s">
         <v>132</v>
       </c>
@@ -19027,7 +19036,7 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="54" t="s">
         <v>65</v>
       </c>
@@ -19035,7 +19044,7 @@
         <v>0.65</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="54" t="s">
         <v>133</v>
       </c>
@@ -19043,7 +19052,7 @@
         <v>0.37</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="54" t="s">
         <v>134</v>
       </c>
@@ -19051,7 +19060,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="54" t="s">
         <v>135</v>
       </c>
@@ -19068,7 +19077,7 @@
       </c>
     </row>
     <row r="34" spans="14:14" ht="51" x14ac:dyDescent="0.2">
-      <c r="N34" s="112" t="s">
+      <c r="N34" s="86" t="s">
         <v>175</v>
       </c>
     </row>
@@ -19261,212 +19270,212 @@
         <v>126</v>
       </c>
       <c r="B2" s="64">
-        <f>'Capacity Factor-Reports'!B2</f>
-        <v>0.65</v>
+        <f>'Capacity Factor-Reports'!C2</f>
+        <v>0.49</v>
       </c>
       <c r="C2" s="64">
         <f>B2</f>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="D2" s="64">
         <f t="shared" ref="D2:AG10" si="0">C2</f>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="E2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="F2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="G2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="H2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="I2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="J2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="K2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="L2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="M2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="N2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="O2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="P2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="Q2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="R2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="S2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="T2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="U2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="V2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="W2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="X2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="Y2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="Z2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="AA2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="AB2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="AC2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="AD2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="AE2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="AF2" s="64">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="AG2" s="79">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="AH2" s="82">
         <f>AG2</f>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="AI2" s="82">
         <f t="shared" ref="AI2:BA16" si="1">AH2</f>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="AJ2" s="82">
         <f t="shared" si="1"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="AK2" s="82">
         <f t="shared" si="1"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="AL2" s="82">
         <f t="shared" si="1"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="AM2" s="82">
         <f t="shared" si="1"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="AN2" s="82">
         <f t="shared" si="1"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="AO2" s="82">
         <f t="shared" si="1"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="AP2" s="82">
         <f t="shared" si="1"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="AQ2" s="82">
         <f t="shared" si="1"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="AR2" s="82">
         <f t="shared" si="1"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="AS2" s="82">
         <f t="shared" si="1"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="AT2" s="82">
         <f t="shared" si="1"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="AU2" s="82">
         <f t="shared" si="1"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="AV2" s="82">
         <f t="shared" si="1"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="AW2" s="82">
         <f t="shared" si="1"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="AX2" s="82">
         <f t="shared" si="1"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="AY2" s="82">
         <f t="shared" si="1"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="AZ2" s="82">
         <f t="shared" si="1"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="BA2" s="82">
         <f t="shared" si="1"/>
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
     </row>
     <row r="3" spans="1:55" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -28391,7 +28400,7 @@
         <v>126</v>
       </c>
       <c r="B2" s="63">
-        <f>'BECF-pre-ret'!B2</f>
+        <f>'Capacity Factor-Reports'!B2</f>
         <v>0.65</v>
       </c>
       <c r="C2" s="63">

</xml_diff>